<commit_message>
PRISME lot 5 (suite) : fiches EDB des 38 divergences fortes, page 2069, notices introuvables
- 33 fiches EDB détaillées + 2 fragments joints (n° 378) archivées et analysées
  (edb/divergences_fortes_fiches.csv, dossiers § H)
- nouvelles datations incertaines : n° 52 (333/358, CLRE), 431 (398/399, CLRE),
  165 (372 conjectural), 220 (381 incertain)
- n° 306 et 378 : textes à vérifier sur l'ICVR
- page EDB 2069, EDCS (nouvelle adresse) et EDH : 6 notices toujours sans second témoin
- registre, journal, chapitre 5.4, Excel et cahier mis à jour

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018MA1py41WVmv44hMs7iE7u
</commit_message>
<xml_diff>
--- a/06_livrables/PRISME_collation_EDCS_EDB.xlsx
+++ b/06_livrables/PRISME_collation_EDCS_EDB.xlsx
@@ -15,18 +15,20 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Registre_consultations" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statistiques" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consuls_lus_restitues" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Faux_consuls_v2" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Divergences_fortes" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Faux_consuls_v2" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Lisez-moi'!$A$1:$B$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Lisez-moi'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Collation'!$A$1:$O$479</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Chrismes_croix'!$A$1:$C$49</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Divergences_dates'!$A$1:$E$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Divergences_dates'!$A$1:$E$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Dossiers'!$A$1:$E$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Registre_consultations'!$A$1:$G$381</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Registre_consultations'!$A$1:$G$389</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Statistiques'!$A$1:$C$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Consuls_lus_restitues'!$A$1:$H$463</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Faux_consuls_v2'!$A$1:$F$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Divergences_fortes'!$A$1:$E$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Faux_consuls_v2'!$A$1:$F$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -446,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -516,41 +518,1068 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Consuls (lot 5)</t>
+          <t>Divergences fortes (lot 5)</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Fondement de l'année de 457 textes à datation directe : A lu 338, B partiel 97, C initiales 2, R restitué 20 ; 30 faux consuls de la v2.0 (feuilles Consuls_lus_restitues, Faux_consuls_v2)</t>
+          <t>38 notices relues sur les fiches EDB détaillées (feuille Divergences_fortes) ; nouvelles datations incertaines : n° 52, 165, 220, 431</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Licences</t>
+          <t>Consuls (lot 5)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>EDB et EDH : CC BY-SA 4.0</t>
+          <t>Fondement de l'année de 457 textes à datation directe : A lu 338, B partiel 97, C initiales 2, R restitué 20 ; 30 faux consuls de la v2.0 (feuilles Consuls_lus_restitues, Faux_consuls_v2)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>Licences</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>EDB et EDH : CC BY-SA 4.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
           <t>Source</t>
         </is>
       </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>PR martinialexisangel-sudo/alexis-angel-martini#1</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B9"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>annee_v2</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>nom_liste_v2</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>forme_dans_le_texte</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>annee_affectee</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>348.0</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Rufinus</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Rufino marito suo</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>époux défunt (dédicataire)</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>349.0</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Euodius</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Eu{u}odius qui vixit annos LXV</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>défunt</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>359.0</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Marcellinus</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>depositus est … Marcellinus</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>défunt (la date consulaire Acindyno et Proculo, 340, est celle de la naissance)</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>362.0</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Eutychianus</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Eutyches pater fecit</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>dédicant (père)</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>105</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>366.0</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Vincentius</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Vincentius / presb(yter)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>défunt, prêtre</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>368.0</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Leontius</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Leontia con[iunx]</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>défunte</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>142</t>
+        </is>
+      </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>PR martinialexisangel-sudo/alexis-angel-martini#1</t>
+          <t>370.0</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Rufinus</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Puer Rufin[us]</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>défunt</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>147</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>371.0</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Constantius</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>ego Cons/tantius compari meae</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>dédicant (époux)</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>155</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>372.0</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Romulus</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Romuliano bene merenti</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>défunt (le second consul lu est Arantheo = Arintheus)</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>166</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>373.0</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Amantius</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Amantio bene mere/nti</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>défunt</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>191</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>376.0</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Eusebius</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Eusebius qui vixit</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>défunt</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>194</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>376.0</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Marcellinus</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Marcellinae quae vi[xit</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>défunte</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>218</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>380.0</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Paulus</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>amoris Pauli[</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>personne nommée dans l’éloge (non consul en 380)</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>247</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>383.0</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Iovianus</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Ioviano karissimo</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>défunt</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>276</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>385.0</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Leontius</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>defunctus Leo/ntius neof&lt;y=I&gt;tus</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>défunt, néophyte</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>281</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>385.0</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Rufinus</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Locus Rufin[ae</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>propriétaire de la tombe</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>309</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>389.0</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Eusebius</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>[domus] aeterna Eusebi</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>défunt ; le consul lu est Timatio (Timasius), absent de la liste v2.0</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>319</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>390.0</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Cerealis</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>C&lt;e=C&gt;r{r}eal(is) bene me(re)nti coniugi</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>dédicant (époux)</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>321</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>390.0</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Philippus</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>administrante Fl(avio) Filippo vir[o clarissimo</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>fonctionnaire nommé dans l’inscription (non consul)</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>321</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>390.0</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Paulus</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Columna Paul(i) a[postol(i)]</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>apôtre Paul</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>352</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>393.0</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Eutychianus</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Eut&lt;y=I&gt;chius sapiens</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>défunt</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>378</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>395.0</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Limenius</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Limenius v]ixit ann[os</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>défunt</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>383</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>395.0</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Amantius</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Dep(ositio) Amanti(a)es(!)</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>défunte</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>387</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>396.0</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Paulus</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>[ad limina Petri et] / Pauli</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>apôtre Paul</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>398</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>397.0</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Paulus</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Paulus qui vixit ann(os) LIIII</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>défunt</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>446</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>400.0</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Vincentius</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Vincentius qui vi(xit)</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>défunt</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>448</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>401.0</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Abundantius</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Depositio Abundanti</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>défunt</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>452</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>401.0</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Theodosius</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Theodosius v(ir) [c(larissimus)</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>défunt ou dédicant, clarissime (non l’empereur)</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>460</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>402.0</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Leontius</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>requiescit Leontia</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>défunte</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>462</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>402.0</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Saturninus</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>[S]aturnino q(ui) v(ixit) (EDB)</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>défunt</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B8"/>
+  <autoFilter ref="A1:F31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -31789,7 +32818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -32033,8 +33062,54 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>EDB17462</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>358</v>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>333 ; 358</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>CLRE p. 631 (cité par l'EDB) : Da[ = Datianus (358) ou Dalmatius (333) ; pierre perdue</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>431</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>EDB27849</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>399</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>398 ; 399</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>CLRE p. 661 : 398 ; Harchadi pour Honorii ; post restitué trop long</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E10"/>
+  <autoFilter ref="A1:E12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -32418,7 +33493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G381"/>
+  <dimension ref="A1:G389"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -45827,8 +46902,268 @@
         </is>
       </c>
     </row>
+    <row r="382">
+      <c r="A382" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B382" s="2" t="inlineStr">
+        <is>
+          <t>Parallel Search web_fetch</t>
+        </is>
+      </c>
+      <c r="C382" s="2" t="inlineStr">
+        <is>
+          <t>https://www.edb.uniba.it/epigraph/{878,12500,17462,20076,20584,22306,24671,24690,24920,25348,27045,27849,28939,28954,29526,30687,31184}</t>
+        </is>
+      </c>
+      <c r="D382" s="2" t="inlineStr">
+        <is>
+          <t>extract_2a473ad4722dd31d0af5b17e43944c1f</t>
+        </is>
+      </c>
+      <c r="E382" s="2" t="inlineStr">
+        <is>
+          <t>17 fiches détaillées lues (fichier edb/fiches/fiches_lot5_*.json)</t>
+        </is>
+      </c>
+      <c r="F382" s="2" t="inlineStr"/>
+      <c r="G382" s="2" t="inlineStr">
+        <is>
+          <t>divergences fortes (lot 5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B383" s="2" t="inlineStr">
+        <is>
+          <t>Parallel Search web_fetch</t>
+        </is>
+      </c>
+      <c r="C383" s="2" t="inlineStr">
+        <is>
+          <t>https://www.edb.uniba.it/epigraph/{31189,31195,31204,31761,31763,33127,33145,33147,35372,35690,39161,39561,39562,39576,40555,42643}</t>
+        </is>
+      </c>
+      <c r="D383" s="2" t="inlineStr">
+        <is>
+          <t>extract_94ec288fff803aad7900323f5f63150a</t>
+        </is>
+      </c>
+      <c r="E383" s="2" t="inlineStr">
+        <is>
+          <t>16 fiches détaillées lues (fichier edb/fiches/fiches_lot5_*.json)</t>
+        </is>
+      </c>
+      <c r="F383" s="2" t="inlineStr"/>
+      <c r="G383" s="2" t="inlineStr">
+        <is>
+          <t>divergences fortes (lot 5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B384" s="2" t="inlineStr">
+        <is>
+          <t>Parallel Search web_fetch</t>
+        </is>
+      </c>
+      <c r="C384" s="2" t="inlineStr">
+        <is>
+          <t>https://www.edb.uniba.it/epigraph/{25442,42793}</t>
+        </is>
+      </c>
+      <c r="D384" s="2" t="inlineStr">
+        <is>
+          <t>extract_7877f47f79170f8a654b222da53a391e</t>
+        </is>
+      </c>
+      <c r="E384" s="2" t="inlineStr">
+        <is>
+          <t>2 fiches lues (fragments joints à ICVR III 8345)</t>
+        </is>
+      </c>
+      <c r="F384" s="2" t="inlineStr"/>
+      <c r="G384" s="2" t="inlineStr">
+        <is>
+          <t>n° 378</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B385" s="2" t="inlineStr">
+        <is>
+          <t>Parallel Search web_fetch</t>
+        </is>
+      </c>
+      <c r="C385" s="2" t="inlineStr">
+        <is>
+          <t>https://www.edb.uniba.it/search/quick/do?page=2069</t>
+        </is>
+      </c>
+      <c r="D385" s="2" t="inlineStr">
+        <is>
+          <t>extract_7877f47f79170f8a654b222da53a391e</t>
+        </is>
+      </c>
+      <c r="E385" s="2" t="inlineStr">
+        <is>
+          <t>page lue ; 20 fiches ; aucune des 6 notices introuvables</t>
+        </is>
+      </c>
+      <c r="F385" s="2" t="inlineStr"/>
+      <c r="G385" s="2" t="inlineStr">
+        <is>
+          <t>notices sans ICUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B386" s="2" t="inlineStr">
+        <is>
+          <t>Parallel Search web_fetch</t>
+        </is>
+      </c>
+      <c r="C386" s="2" t="inlineStr">
+        <is>
+          <t>https://edcs.hist.uzh.ch/search?citation={CIL 06, 08405 ; AE 2016, 00170 ; AE 2010, 00207 ; AE 2003, 00216 ; AE 1994, 00263 ; Carletti-2008, 00177}</t>
+        </is>
+      </c>
+      <c r="D386" s="2" t="inlineStr">
+        <is>
+          <t>extract_01b3d2af2bcd96e4c132255fcf837824</t>
+        </is>
+      </c>
+      <c r="E386" s="2" t="inlineStr">
+        <is>
+          <t>nouvelle adresse de l'EDCS (uzh.ch) accessible par le relais ; 5 références trouvées (1 résultat chacune), la recherche « Carletti-2008 » ne renvoie rien</t>
+        </is>
+      </c>
+      <c r="F386" s="2" t="inlineStr"/>
+      <c r="G386" s="2" t="inlineStr">
+        <is>
+          <t>6 notices introuvables</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B387" s="2" t="inlineStr">
+        <is>
+          <t>Parallel Search web_fetch</t>
+        </is>
+      </c>
+      <c r="C387" s="2" t="inlineStr">
+        <is>
+          <t>https://edcs.hist.uzh.ch/monument/{18200424,75200321,59400075,29900387,02700284,71500011}</t>
+        </is>
+      </c>
+      <c r="D387" s="2" t="inlineStr">
+        <is>
+          <t>extract_4f461b8de1a6246aff302b5d0a259631</t>
+        </is>
+      </c>
+      <c r="E387" s="2" t="inlineStr">
+        <is>
+          <t>6 fiches EDCS lues ; aucune équivalence ICUR ; texte identique à la v2.0 ; photo signalée pour EDCS-71500011 seulement</t>
+        </is>
+      </c>
+      <c r="F387" s="2" t="inlineStr"/>
+      <c r="G387" s="2" t="inlineStr">
+        <is>
+          <t>6 notices introuvables</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B388" s="2" t="inlineStr">
+        <is>
+          <t>git grep (dump EDH local)</t>
+        </is>
+      </c>
+      <c r="C388" s="2" t="inlineStr">
+        <is>
+          <t>références AE 2010 207 ; AE 2003 216 ; AE 1994 263 ; AE 2016 170 ; CIL VI 8405 ; « Martiel »</t>
+        </is>
+      </c>
+      <c r="D388" s="2" t="inlineStr"/>
+      <c r="E388" s="2" t="inlineStr">
+        <is>
+          <t>aucune correspondance (seuls des faux positifs AE 2010 1207 etc.)</t>
+        </is>
+      </c>
+      <c r="F388" s="2" t="inlineStr"/>
+      <c r="G388" s="2" t="inlineStr">
+        <is>
+          <t>6 notices introuvables</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B389" s="2" t="inlineStr">
+        <is>
+          <t>Parallel Search web_search</t>
+        </is>
+      </c>
+      <c r="C389" s="2" t="inlineStr">
+        <is>
+          <t>edb.uniba.it Martielis numerarius ; « Eros et Leo et Setema » ; Criscentinae … Priscus ; numerarius vicariae sedis</t>
+        </is>
+      </c>
+      <c r="D389" s="2" t="inlineStr">
+        <is>
+          <t>search_ac0db094919b0c8b2c8f3d1ebf78d479</t>
+        </is>
+      </c>
+      <c r="E389" s="2" t="inlineStr">
+        <is>
+          <t>aucun résultat pertinent</t>
+        </is>
+      </c>
+      <c r="F389" s="2" t="inlineStr"/>
+      <c r="G389" s="2" t="inlineStr">
+        <is>
+          <t>6 notices introuvables</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G381"/>
+  <autoFilter ref="A1:G389"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -47857,7 +49192,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Da[tiani : 2 lettres gravées ; Cerealis entièrement restitué.</t>
+          <t>Da[tiani : 2 lettres gravées ; Cerealis entièrement restitué. Fiche EDB17462 (d'après CLRE p. 631) : Da[ peut aussi être Dalmatius (333) ; date incertaine 333/358.</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -51666,10 +53001,14 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="G162" s="2" t="inlineStr"/>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="G162" s="2" t="inlineStr">
+        <is>
+          <t>Mo]dest[o : 4 lettres gravées (« dest ») ; Arintheus restitué. Fiche EDB40555 : date 300-399 ; l'année 372 est une hypothèse de Ferrua.</t>
+        </is>
+      </c>
       <c r="H162" s="2" t="inlineStr">
         <is>
           <t>p]ace VII [3] / [3 Mo]dest[o et Arintheo cons(ulibus?)</t>
@@ -53476,10 +54815,14 @@
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="G215" s="2" t="inlineStr"/>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="G215" s="2" t="inlineStr">
+        <is>
+          <t>Euch]erio : 4 lettres gravées (« erio ») ; fiche EDB30687 : Val]erio, Gal]erio, Neot]erio, Ast]erio possibles ; date 381 incertaine.</t>
+        </is>
+      </c>
       <c r="H215" s="2" t="inlineStr">
         <is>
           <t>[3]ECIM[3] / [3]NOM[3] / [3 Fl(avio) Sygario et Fl(avio) Euch]erio [vv(iris) cc(larissimis) cons(ulibus)</t>
@@ -62026,15 +63369,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
     <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="35" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -62045,992 +63387,1053 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>annee_v2</t>
+          <t>edb_id</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>nom_liste_v2</t>
+          <t>cause</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>forme_dans_le_texte</t>
+          <t>constat (fiche EDB détaillée, lue le 14/10/2026)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>role</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>annee_affectee</t>
+          <t>consequence</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>348.0</t>
+          <t>EDB31184</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Rufinus</t>
+          <t>notation</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Rufino marito suo</t>
+          <t>Même texte. L'EDB garde la graphie de la pierre (bixit, birginia), l'EDCS la corrige (&lt;v=B&gt;). L'EDB décrit un chrisme final. Supports bibliographiques : Di Stefano Manzella 1997 (avec photo), Carletti 1986a n. 89.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>époux défunt (dédicataire)</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+          <t>aucune sur la date (341) ; chrisme à compter</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>349.0</t>
+          <t>EDB39161</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Euodius</t>
+          <t>restitutions divergentes</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Eu{u}odius qui vixit annos LXV</t>
+          <t>L'EDCS restitue beaucoup plus : [c(larissimae)] m(emoriae) f(eminae) venit [ante annos d]uos, cu[m compare sua Lea(?)], et Lea vixit. L'EDB lit m(onumentum?) f(ecerunt?) ++++, cu[m ---]uos, et dies XX (EDCS : XXI). Sarcophage, ICVR IV 10851 = CIL VI 9237.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>défunt</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+          <t>date inchangée (347) ; ne pas exploiter Lea, c.m.f. ni les durées sans contrôle ICVR</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>51</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>359.0</t>
+          <t>EDB31763</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Marcellinus</t>
+          <t>ligne absente de l'EDCS</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>depositus est … Marcellinus</t>
+          <t>EDB (selon Lega 2000) : [--- Datiano et C]aereale [consulibus? ---]. Déjà traité (§ D, A016).</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>défunt (la date consulaire Acindyno et Proculo, 340, est celle de la naissance)</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+          <t>déjà intégré</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>52</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>362.0</t>
+          <t>EDB17462</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Eutychianus</t>
+          <t>datation contestée</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Eutyches pater fecit</t>
+          <t>Note EDB (Vilella, d'après CLRE p. 631) : la lecture Da[tiano et Cereale] de Silvagni est incertaine, car Dalmatius, consul en 333 avec Zenophilus, commence aussi par DA. Pierre perdue. Transcription EDB différente de l'ICVR.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>dédicant (père)</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+          <t>date incertaine 333/358 ; si 333, hors corpus</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>73</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>366.0</t>
+          <t>EDB31189</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Vincentius</t>
+          <t>restitutions divergentes</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Vincentius / presb(yter)</t>
+          <t>Carmen d'Eleuteria : restitutions différentes (déjà traité). L'EDB décrit palmes, soleil, chrisme, croix gammée, alpha et oméga.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>défunt, prêtre</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+          <t>déjà intégré</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>125</t>
+          <t>98</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>368.0</t>
+          <t>EDB20076</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Leontius</t>
+          <t>datation</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Leontia con[iunx]</t>
+          <t>Déjà traité : Severinus lu ; 461 ou 482 (CLRE p. 680).</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>défunte</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+          <t>hors corpus (déjà)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>113</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>370.0</t>
+          <t>EDB31195</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Rufinus</t>
+          <t>notation</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Puer Rufin[us]</t>
+          <t>Même texte (lecture Lega 2000).</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>défunt</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+          <t>aucune</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>147</t>
+          <t>115</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>371.0</t>
+          <t>EDB33127</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Constantius</t>
+          <t>notation</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>ego Cons/tantius compari meae</t>
+          <t>Même texte ; non(is) / non(as).</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>dédicant (époux)</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+          <t>aucune</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>155</t>
+          <t>123</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>372.0</t>
+          <t>EDB24921</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Romulus</t>
+          <t>lecture divergente</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Romuliano bene merenti</t>
+          <t>Déjà traité (A016) : obiit (EDCS) contre [Lupicin]o et Iovi[no] (EDB).</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>défunt (le second consul lu est Arantheo = Arintheus)</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+          <t>déjà intégré</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>166</t>
+          <t>134</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>373.0</t>
+          <t>EDB24671</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Amantius</t>
+          <t>structure et lecture</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Amantio bene mere/nti</t>
+          <t>Grande dalle (105 x 190 x 15) en plusieurs textes (a, b…), remployée en morceaux dans un mur (Marucchi 1914, cité par l'EDB). Photo PCAS signalée. Lecture du nom : Ca[t]afronies (EDCS) / Ca[l]ifronies (EDB). Date EDB « 350-399 ; 369 ».</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>défunt</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+          <t>date 369 portée par une partie seulement du monument ; à vérifier sur ICVR III 8148</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>152</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>376.0</t>
+          <t>EDB39561</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Eusebius</t>
+          <t>restitutions divergentes (texte métrique)</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Eusebius qui vixit</t>
+          <t>Marce na[---] (EDB) / Marcena (EDCS) ; [cor]p&lt;o&gt;re demptus (EDB) / PQ redemptus (EDCS). Dalle perdue, connue par de Rossi 1864 et le dessin d'IC I.</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>défunt</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+          <t>date 371 inchangée</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>194</t>
+          <t>153</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>376.0</t>
+          <t>EDB39562</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Marcellinus</t>
+          <t>restitution EDCS</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Marcellinae quae vi[xit</t>
+          <t>L'EDB ne restitue pas Gratien : +++++++CE+[---] / et Probo c[onsulibus]. L'EDCS restitue [Gratiano Aug(usto) II].</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>défunte</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+          <t>date 371 par Probus seul (lu)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>218</t>
+          <t>165</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>380.0</t>
+          <t>EDB40555</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Paulus</t>
+          <t>datation conjecturale</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>amoris Pauli[</t>
+          <t>EDB : [--- in p]ace VII / [---]dest[---] ; date 300-399. Note : « Ferrua putat esse data consulatus Modesti et Arinthei a. 372 ». L'année 372 repose sur la seule séquence « dest ».</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>personne nommée dans l’éloge (non consul en 380)</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+          <t>datation conjecturale (372 = hypothèse de Ferrua)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>247</t>
+          <t>180</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>383.0</t>
+          <t>EDB31761</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Iovianus</t>
+          <t>ligne absente / lecture Lega</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Ioviano karissimo</t>
+          <t>Déjà traité (A016).</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>défunt</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+          <t>déjà intégré</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>276</t>
+          <t>193</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>385.0</t>
+          <t>EDB878</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Leontius</t>
+          <t>notation</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>defunctus Leo/ntius neof&lt;y=I&gt;tus</t>
+          <t>Même texte ; consul&lt;ibus=ATV&gt; (EDCS) / consulatu (EDB). Chrisme avec alpha et oméga.</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>défunt, néophyte</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+          <t>aucune sur la date</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>281</t>
+          <t>214</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>385.0</t>
+          <t>EDB33145</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Rufinus</t>
+          <t>lignes absentes de l'EDCS</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Locus Rufin[ae</t>
+          <t>Déjà traité (A016) : formule consulaire de 380 transmise par l'EDB.</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>propriétaire de la tombe</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+          <t>déjà intégré</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>309</t>
+          <t>220</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>389.0</t>
+          <t>EDB30687</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Eusebius</t>
+          <t>datation incertaine</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>[domus] aeterna Eusebi</t>
+          <t>EDB : [--- et Fl(avio) Euch?]erio, avec la note « there are other possible readings: Val]erio, Gal]erio, Neot]erio, Ast]erio ». Seul « erio » est lu. L'EDCS restitue Sygario et Euch]erio sans réserve.</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>défunt ; le consul lu est Timatio (Timasius), absent de la liste v2.0</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+          <t>date 381 incertaine (Neoterio = 390 possible)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>319</t>
+          <t>222</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>390.0</t>
+          <t>EDB33147</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Cerealis</t>
+          <t>lecture ICVR I 1209</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>C&lt;e=C&gt;r{r}eal(is) bene me(re)nti coniugi</t>
+          <t>Même texte pour la date (Fl(avio) Sy[agrio). L'EDB suit ICVR I 1209 et non I 1396 (Ferrua 1979b).</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>dédicant (époux)</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+          <t>aucune ; niveau R maintenu</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>321</t>
+          <t>231</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>390.0</t>
+          <t>EDB31204</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Philippus</t>
+          <t>lecture Lega</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>administrante Fl(avio) Filippo vir[o clarissimo</t>
+          <t>Antino (EDB, d'après Lega) / Ant&lt;o=I&gt;n(i)o (EDCS) ; d(iebus) / d(epositus).</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>fonctionnaire nommé dans l’inscription (non consul)</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+          <t>date 382 inchangée</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>321</t>
+          <t>290</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>390.0</t>
+          <t>EDB39576</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Paulus</t>
+          <t>restitution EDCS</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Columna Paul(i) a[postol(i)]</t>
+          <t>L'EDB s'arrête à Ho[norio ---]. Note de Ferrua (via l'EDB) : seul le premier consulat d'Honorius (386) le nomme Flavius. L'EDCS restitue n(obilissimo) p(uero) et Fl(avio) Euodio.</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>apôtre Paul</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+          <t>date 386 argumentée (Fl. + Ho-), mais restituée</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>352</t>
+          <t>306</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>393.0</t>
+          <t>EDB27045</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Eutychianus</t>
+          <t>ligne absente de l'EDB ?</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Eut&lt;y=I&gt;chius sapiens</t>
+          <t>L'EDCS donne une ligne « et innocentiae optimique propositi Maximilla virgo ancilla dei civis Pannonia qu(a)e » absente du texte EDB (qui passe de « Mirae fide〈i〉 » à « vixit annis »). Sarcophage, Platonia de Saint-Sébastien, ICVR V 13355 ; Mazzoleni 2015, 167.</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>défunt</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+          <t>à vérifier sur ICVR V 13355 : la ligne contient « virgo ancilla dei »</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>378</t>
+          <t>313</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>395.0</t>
+          <t>EDB39579</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Limenius</t>
+          <t>structure</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Limenius v]ixit ann[os</t>
+          <t>Déjà traité (A009).</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>défunt</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+          <t>déjà intégré</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>383</t>
+          <t>314</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>395.0</t>
+          <t>EDB39579</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Amantius</t>
+          <t>structure</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Dep(ositio) Amanti(a)es(!)</t>
+          <t>Déjà traité (A009).</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>défunte</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+          <t>déjà intégré</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>387</t>
+          <t>321</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>396.0</t>
+          <t>EDB42643</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Paulus</t>
+          <t>structure</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>[ad limina Petri et] / Pauli</t>
+          <t>Colonne de Saint-Paul, trois textes (a, b, c). Lecture de Filippi 2000 ; AE 2000, 187 ; EDR074191.</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>apôtre Paul</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+          <t>date 390 inchangée</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>398</t>
+          <t>326</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>397.0</t>
+          <t>EDB24920</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Paulus</t>
+          <t>restitution EDB</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Paulus qui vixit ann(os) LIIII</t>
+          <t>Déjà traité (A016) : ]eute[ seul lu.</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>défunt</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+          <t>déjà intégré</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>446</t>
+          <t>352</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>400.0</t>
+          <t>EDB28954</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Vincentius</t>
+          <t>notation</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Vincentius qui vi(xit)</t>
+          <t>Même texte ; [con]s(ulatu) Theodosi Aug(usti) III et Eugen-/[i] (EDB). Note de de Rossi sur la fin. Pierre perdue.</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>défunt</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+          <t>date 393 inchangée</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>448</t>
+          <t>378</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>401.0</t>
+          <t>EDB25348</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Abundantius</t>
+          <t>monument composite</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Depositio Abundanti</t>
+          <t>La fiche EDB (ICVR III 8345) ne contient que le début du poème. Elle est à joindre à ICVR III 8274c (EDB25442) et 8387v (EDB42793) ; selon l'EDB, 8345 est formé de quatre fragments. Aucune des trois fiches ne contient la formule [Olybrio et Pro]bino ni la généalogie (Limenius presbyter, Marcellus episcopus, Ursinus Albanensis) du texte EDCS. Date EDB : 390-424.</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>défunt</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+          <t>date 395 portée par une partie non retrouvée dans l'EDB ; à vérifier sur ICVR III 8345</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>452</t>
+          <t>382</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>401.0</t>
+          <t>EDB20584</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Theodosius</t>
+          <t>notation</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Theodosius v(ir) [c(larissimus)</t>
+          <t>Même texte ; l'EDCS ajoute « // [Pa]nthagate » absent de l'EDB.</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>défunt ou dédicant, clarissime (non l’empereur)</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+          <t>aucune sur la date</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>460</t>
+          <t>393</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>402.0</t>
+          <t>EDB39590</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Leontius</t>
+          <t>structure</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>requiescit Leontia</t>
+          <t>Déjà traité (A010).</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>défunte</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+          <t>déjà intégré</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
+          <t>394</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>EDB39590</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>structure</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Déjà traité (A010).</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>déjà intégré</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>397</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>EDB35690</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>lecture</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Ṛọṃạṇ[---] (EDB) / ]romi[ (EDCS) ; restitution métrique de l'EDB. Pierre perdue ; CIL VI 39147a ; ICVR X 27324.</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>date 397 inchangée</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>EDB29526</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>notation et signes</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Même texte ; l'EDB décrit un chrisme, deux croix monogrammatiques (dont une en couronne) et un oiseau tenant un rameau d'olivier. Notes : VIIIX kal. mart. corrigé par Diehl en prid. id. Febr. ; « Pascasius » n'est pas un évêque de Rome connu (Diehl).</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>date 397 inchangée ; jour du mois douteux</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>431</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>EDB27849</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>datation divergente</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>EDB date « 398 ; 399 ». Notes : Harchadi pour Honorii (erreur du lapicide déjà signalée par Muratori et Silvagni) ; CLRE p. 661 attribue l'inscription à 398, car « post » restitué serait trop long et le p.c. si tard en 399 est sans exemple. La v2.0 retient 399.</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>divergence de date nouvelle : 398 (CLRE) / 399 (v2.0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>435</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>EDB22306</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>restitution EDB</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Déjà traité (A016).</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>déjà intégré</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>445</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>EDB24690</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>ligne absente de l'EDCS</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Déjà traité (A016). Note de Felle : les lettres BA[silica] sont visibles sur la photo PCAS mais pas sur l'image de Marucchi 1914.</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>déjà intégré</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>447</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>EDB12500</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>lignes absentes de l'EDCS</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Déjà traité (A016) : 10 lignes dans l'EDB, 5 dans l'EDCS. Conservation : Museo Nazionale Romano, Terme di Diocleziano.</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>déjà intégré</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
           <t>462</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>402.0</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>Saturninus</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>[S]aturnino q(ui) v(ixit) (EDB)</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>défunt</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>non (l’année repose sur l’autre paire ou le collègue)</t>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>EDB35372</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>lecture</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Déjà vu (§ G) : Saturnino est le défunt ; l'EDB lit e̲t̲ H̲o̲n̲o̲r̲[io] (lettres vues par un éditeur antérieur).</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>date 402 inchangée</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>470</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>EDB28939</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>notation</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Même texte ; Rumorido (EDB) / Rumordio (EDCS). L'EDB décrit une orante et signale l'emprunt virgilien du v. 7 (Aen. VI 429 ; XI 28).</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>aucune sur la date ; citation de Virgile à exploiter</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F31"/>
+  <autoFilter ref="A1:E39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>